<commit_message>
Customer list +10% on shells; labour at $280/day as Div 11.01
Strip factory-net and KDK cost language. Distributor 10% now comes
off the marked-up KDK list. Pad crew table uses KDK selling rates.
</commit_message>
<xml_diff>
--- a/public/CASA100_BOQ_worksheet.xlsx
+++ b/public/CASA100_BOQ_worksheet.xlsx
@@ -8,17 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11.01 vs China crew" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Div 11.01 labour" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOQ lines" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Shell vs add-ons" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Cover'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'11.01 vs China crew'!$1:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'BOQ lines'!$A$3:$O$47</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="2">'BOQ lines'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Shell vs add-ons'!$1:$3</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -56,10 +50,6 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="008A4B08"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="001F4A3A"/>
     </font>
     <font>
@@ -74,6 +64,10 @@
       <color rgb="001F4A3A"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008A4B08"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -81,11 +75,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F4E8C8"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -102,6 +91,11 @@
         <fgColor rgb="00E8EEE8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4E8C8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -115,44 +109,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -518,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="72" customWidth="1" min="1" max="1"/>
@@ -528,7 +521,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CASA 100 — BOQ worksheet (internal)</t>
+          <t>CASA 100 — BOQ worksheet</t>
         </is>
       </c>
     </row>
@@ -540,26 +533,26 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Do not circulate until numbers are signed off. Working draft, not a contract.</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Working draft for government review — not a contract.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Headline</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>USD</t>
         </is>
@@ -571,8 +564,8 @@
           <t>Full village all-in (no extra civil)</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>7616796.72</v>
+      <c r="B8" s="4" t="n">
+        <v>7832399.69</v>
       </c>
     </row>
     <row r="9">
@@ -581,8 +574,8 @@
           <t>Works</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
-        <v>6684919.01</v>
+      <c r="B9" s="4" t="n">
+        <v>6874144.01</v>
       </c>
     </row>
     <row r="10">
@@ -591,8 +584,8 @@
           <t>Contingency 8%</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>534793.52</v>
+      <c r="B10" s="4" t="n">
+        <v>549931.52</v>
       </c>
     </row>
     <row r="11">
@@ -601,100 +594,74 @@
           <t>PM 5.5%</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>397084.19</v>
+      <c r="B11" s="4" t="n">
+        <v>408324.15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11.01 assembly this mix</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
+          <t>Div 11.01 assembly this mix</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
         <v>192080</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>11.01 average / home</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
+          <t>Div 11.01 average / home</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
         <v>1920.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4 Chinese workers at 20 homes (factory sheet, incl. travel)</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>2616</v>
+          <t>Div 11.01 labour / 2-bed (4 workers × 2 days × $280)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>2240</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4 Chinese workers at 100 homes (factory sheet, incl. travel)</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>875.2</v>
+          <t>20 homes, labour + travel / home</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>2736</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>On-site only: 4 × 2 days × $220</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n">
-        <v>1760</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>11.01 2-bed / 3-bed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>2240</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>IMPORTANT</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>11.01 and the 4-worker China sheet are the SAME pad assembly. Do not add them. 11.01 stays in the all-in ($280/day Greython/Maatern method). The China sheet is factory-net $220/day plus a one-time $43,520 travel lump. At 20 homes that averages $2,616/home — same band as 11.01 $2,240 on a 2-bed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
+          <t>100 homes, labour + travel / home</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>995.2</v>
+      </c>
+    </row>
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Div 11.01 = labour to assemble the home on the pad. Do not add the travel table on top of Div 11.01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A20:B22"/>
+    <mergeCell ref="A18:B19"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LCASA 100 BOQ worksheet · internal</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
 
@@ -704,67 +671,66 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pad assembly — BOQ 11.01 vs factory-net 4 Chinese workers</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Factory arithmetic: travel $43,520 + (homes ÷ 2) × 4 × $220. Net, no KDK commission. 4 workers, 2 days per home.</t>
+          <t>Division 11.01 — assembling the home on the pad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>A 2-bed home: four workers, two days, $280 per worker-day = $2,240. Travel for four is a one-time $43,520. Do not add this table on top of Div 11.01.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>BOQ 11.01 (priced in the all-in)</t>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Div 11.01 in the all-in</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Style</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Hours</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Days</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>$280/day amount / home</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Campaign 11.01</t>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Labour / home</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Campaign Div 11.01</t>
         </is>
       </c>
     </row>
@@ -783,10 +749,10 @@
       <c r="D6" t="n">
         <v>4.2</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="4" t="n">
         <v>1176</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="4" t="n">
         <v>35280</v>
       </c>
     </row>
@@ -805,10 +771,10 @@
       <c r="D7" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="4" t="n">
         <v>2240</v>
       </c>
-      <c r="F7" s="5" t="n">
+      <c r="F7" s="4" t="n">
         <v>100800</v>
       </c>
     </row>
@@ -827,15 +793,15 @@
       <c r="D8" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="4" t="n">
         <v>2240</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="4" t="n">
         <v>56000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Campaign total</t>
         </is>
@@ -843,56 +809,41 @@
       <c r="B9" t="n">
         <v>100</v>
       </c>
-      <c r="F9" s="10" t="n">
+      <c r="F9" s="4" t="n">
         <v>192080</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Average / home</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>1920.8</v>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Factory-net 4 Chinese workers (NOT added to 11.01)</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Labour + one-time travel (KDK price — same work as Div 11.01, travel spread)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Homes</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Travel (4 workers)</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>On-site labour</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Factory-net total</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>KDK total</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Per home</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>vs 11.01 avg</t>
         </is>
       </c>
     </row>
@@ -900,80 +851,68 @@
       <c r="A14" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="4" t="n">
         <v>43520</v>
       </c>
-      <c r="C14" s="5" t="n">
-        <v>4400</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>47920</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>4792</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>2871.2</v>
+      <c r="C14" s="4" t="n">
+        <v>5600</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>49120</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>4912</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="A15" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="9" t="n">
         <v>43520</v>
       </c>
-      <c r="C15" s="12" t="n">
-        <v>8800</v>
-      </c>
-      <c r="D15" s="12" t="n">
-        <v>52320</v>
-      </c>
-      <c r="E15" s="12" t="n">
-        <v>2616</v>
-      </c>
-      <c r="F15" s="12" t="n">
-        <v>695.2</v>
+      <c r="C15" s="9" t="n">
+        <v>11200</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>54720</v>
+      </c>
+      <c r="E15" s="9" t="n">
+        <v>2736</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
         <v>50</v>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="4" t="n">
         <v>43520</v>
       </c>
-      <c r="C16" s="5" t="n">
-        <v>22000</v>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>65520</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>1310.4</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>-610.3999999999999</v>
+      <c r="C16" s="4" t="n">
+        <v>28000</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>71520</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>1430.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>100</v>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="4" t="n">
         <v>43520</v>
       </c>
-      <c r="C17" s="5" t="n">
-        <v>44000</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>87520</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>875.2</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>-1045.6</v>
+      <c r="C17" s="4" t="n">
+        <v>56000</v>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>99520</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>995.2</v>
       </c>
     </row>
     <row r="18">
@@ -982,173 +921,34 @@
           <t>This mix (100)</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="4" t="n">
         <v>43520</v>
       </c>
-      <c r="C18" s="5" t="n">
-        <v>44000</v>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>87520</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>875.2</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>-1045.6</v>
+      <c r="C18" s="4" t="n">
+        <v>56000</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>99520</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>995.2</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>On-site only (no travel): 4 workers × 2 days × $220</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>1760</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Greython / Maatern day rate used in 11.01</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Factory-net day rate</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>First two homes — 2 Chinese + 2 Belizean helpers (7–10 days)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Chinese side (user figure) / home</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="n">
-        <v>11000</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Chinese travel (2 workers × $10,000)</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="n">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Chinese site 7–10 days (range)</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="n">
-        <v>23080</v>
-      </c>
-      <c r="F28" s="5" t="n">
-        <v>24400</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>After training — recommended CASA 100 ramp (first 2 trainer pads, then Belizean-majority)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>First two homes (Chinese, user figure)</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="n">
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Belizean helpers on first two (est.)</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="n">
-        <v>1292</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Remaining 98 homes at mixed pad rate</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="n">
-        <v>86051.84</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Ramp total</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="n">
-        <v>109343.84</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Ramp / home</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="n">
-        <v>1093.4384</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>11.01 this mix (kept in the all-in)</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>192080</v>
-      </c>
-    </row>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>First two homes: two Chinese trainers + two Belizean helpers, 7–10 days. Then Belizean crews take over for 12 months or longer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A20:E21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LCASA 100 BOQ worksheet · internal</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
 
@@ -1185,107 +985,107 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Division</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>In price?</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Rate 1-bed</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Rate 2-bed</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Rate 3-bed</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>Amt 1-bed ×30</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Amt 2-bed ×45</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Amt 3-bed ×25</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Project (in price)</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Full amount (if on)</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Container homes</t>
         </is>
       </c>
-      <c r="C4" s="13" t="n"/>
-      <c r="D4" s="13" t="n"/>
-      <c r="E4" s="13" t="n"/>
-      <c r="F4" s="13" t="n"/>
-      <c r="G4" s="13" t="n"/>
-      <c r="H4" s="13" t="n"/>
-      <c r="I4" s="13" t="n"/>
-      <c r="J4" s="13" t="n"/>
-      <c r="K4" s="13" t="n"/>
-      <c r="L4" s="13" t="n"/>
-      <c r="M4" s="13" t="n"/>
-      <c r="N4" s="13" t="n"/>
-      <c r="O4" s="13" t="n"/>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
+      <c r="I4" s="10" t="n"/>
+      <c r="J4" s="10" t="n"/>
+      <c r="K4" s="10" t="n"/>
+      <c r="L4" s="10" t="n"/>
+      <c r="M4" s="10" t="n"/>
+      <c r="N4" s="10" t="n"/>
+      <c r="O4" s="10" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1298,9 +1098,9 @@
           <t>Container homes</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Basic shell module — list price, unfurnished (FOB China port)</t>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Basic shell module — KDK list, unfurnished (FOB China port)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1318,33 +1118,33 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n">
-        <v>15850</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>23100</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>23500</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>475500</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>1039500</v>
-      </c>
-      <c r="L5" s="5" t="n">
-        <v>587500</v>
-      </c>
-      <c r="M5" s="5" t="n">
-        <v>2102500</v>
-      </c>
-      <c r="N5" s="5" t="n">
-        <v>2102500</v>
-      </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
-          <t>Basic SHELL: steel frames, walls, insulated roof, doors, windows, house lights/sockets/DB, kitchen cabinet + sink + faucet, ceramic toilet, wash-basin, glass shower, bathroom pipework. Unfurnished. FOB China — no ocean, no inland. NOT in the shell: split air, solar, range, fridge, furniture, gas stove, pads, village works.</t>
+      <c r="G5" s="4" t="n">
+        <v>17435</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>25410</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>25850</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>523050</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>1143450</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>646250</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>2312750</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>2312750</v>
+      </c>
+      <c r="O5" s="5" t="inlineStr">
+        <is>
+          <t>KDK list for the basic SHELL (FOB China). 10% campaign/distributor discount is 01.02. Kitchen, toilet, shower and house electrics are in the box. Split air, solar, range, fridge, furniture, pads and village works are not.</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1159,7 @@
           <t>Container homes</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Belize set-aside / distributor — 10% of shell list</t>
         </is>
@@ -1379,60 +1179,60 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>-1585</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>-2310</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>-2350</v>
-      </c>
-      <c r="J6" s="5" t="n">
-        <v>-47550</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>-103950</v>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>-58750</v>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>-210250</v>
-      </c>
-      <c r="N6" s="5" t="n">
-        <v>-210250</v>
-      </c>
-      <c r="O6" s="7" t="inlineStr">
-        <is>
-          <t>On the shell list only. 10% of factory list. KDK Hong Kong path = discount to the Government. Licensed Belizean distributor path = set-aside / seller margin. Not on slabs, solar, or village works.</t>
+      <c r="G6" s="4" t="n">
+        <v>-1743.5</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>-2541</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>-2585</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>-52305</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>-114345</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>-64625</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>-231275</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>-231275</v>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>On the shell list only. 10% of KDK list. KDK Hong Kong path = discount to the Government. Licensed Belizean distributor path = set-aside / seller margin. Not on slabs, solar, or village works.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Logistics</t>
         </is>
       </c>
-      <c r="C7" s="13" t="n"/>
-      <c r="D7" s="13" t="n"/>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n"/>
-      <c r="H7" s="13" t="n"/>
-      <c r="I7" s="13" t="n"/>
-      <c r="J7" s="13" t="n"/>
-      <c r="K7" s="13" t="n"/>
-      <c r="L7" s="13" t="n"/>
-      <c r="M7" s="13" t="n"/>
-      <c r="N7" s="13" t="n"/>
-      <c r="O7" s="13" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="10" t="n"/>
+      <c r="M7" s="10" t="n"/>
+      <c r="N7" s="10" t="n"/>
+      <c r="O7" s="10" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1445,7 +1245,7 @@
           <t>Logistics</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Ocean freight, China → Belize ($19,000 per 40HQ ÷ units/container)</t>
         </is>
@@ -1465,31 +1265,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="4" t="n">
         <v>6333.333333333333</v>
       </c>
-      <c r="H8" s="5" t="n">
+      <c r="H8" s="4" t="n">
         <v>9500</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="I8" s="4" t="n">
         <v>10439.56043956044</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="J8" s="4" t="n">
         <v>190000</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="4" t="n">
         <v>427500</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="L8" s="4" t="n">
         <v>260989.010989011</v>
       </c>
-      <c r="M8" s="5" t="n">
+      <c r="M8" s="4" t="n">
         <v>878489.010989011</v>
       </c>
-      <c r="N8" s="5" t="n">
+      <c r="N8" s="4" t="n">
         <v>878489.010989011</v>
       </c>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="O8" s="5" t="inlineStr">
         <is>
           <t>Load factors 3 / 2 / 1.82 per 40HQ. Full-container campaign — no lone-home penalty.</t>
         </is>
@@ -1506,7 +1306,7 @@
           <t>Logistics</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Inland delivery to site gate + duties/taxes (HS 9406.20)</t>
         </is>
@@ -1526,60 +1326,60 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="4" t="n">
         <v>3200</v>
       </c>
-      <c r="H9" s="5" t="n">
+      <c r="H9" s="4" t="n">
         <v>3200</v>
       </c>
-      <c r="I9" s="5" t="n">
+      <c r="I9" s="4" t="n">
         <v>3200</v>
       </c>
-      <c r="J9" s="5" t="n">
+      <c r="J9" s="4" t="n">
         <v>96000</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="K9" s="4" t="n">
         <v>144000</v>
       </c>
-      <c r="L9" s="5" t="n">
+      <c r="L9" s="4" t="n">
         <v>80000</v>
       </c>
-      <c r="M9" s="5" t="n">
+      <c r="M9" s="4" t="n">
         <v>320000</v>
       </c>
-      <c r="N9" s="5" t="n">
+      <c r="N9" s="4" t="n">
         <v>320000</v>
       </c>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>Moonlight Bay carried $5,000/home for two units. Convoy rate for 100.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Foundations &amp; anchoring</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n"/>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
-      <c r="I10" s="13" t="n"/>
-      <c r="J10" s="13" t="n"/>
-      <c r="K10" s="13" t="n"/>
-      <c r="L10" s="13" t="n"/>
-      <c r="M10" s="13" t="n"/>
-      <c r="N10" s="13" t="n"/>
-      <c r="O10" s="13" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="n"/>
+      <c r="J10" s="10" t="n"/>
+      <c r="K10" s="10" t="n"/>
+      <c r="L10" s="10" t="n"/>
+      <c r="M10" s="10" t="n"/>
+      <c r="N10" s="10" t="n"/>
+      <c r="O10" s="10" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1592,7 +1392,7 @@
           <t>Foundations &amp; anchoring</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Concrete slab + excavation + house MEP stub-up</t>
         </is>
@@ -1612,31 +1412,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="4" t="n">
         <v>11500</v>
       </c>
-      <c r="H11" s="5" t="n">
+      <c r="H11" s="4" t="n">
         <v>12500</v>
       </c>
-      <c r="I11" s="5" t="n">
+      <c r="I11" s="4" t="n">
         <v>13000</v>
       </c>
-      <c r="J11" s="5" t="n">
+      <c r="J11" s="4" t="n">
         <v>345000</v>
       </c>
-      <c r="K11" s="5" t="n">
+      <c r="K11" s="4" t="n">
         <v>562500</v>
       </c>
-      <c r="L11" s="5" t="n">
+      <c r="L11" s="4" t="n">
         <v>325000</v>
       </c>
-      <c r="M11" s="5" t="n">
+      <c r="M11" s="4" t="n">
         <v>1232500</v>
       </c>
-      <c r="N11" s="5" t="n">
+      <c r="N11" s="4" t="n">
         <v>1232500</v>
       </c>
-      <c r="O11" s="7" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr">
         <is>
           <t>Moonlight Bay $20,000/home. Campaign crew, government spec slab-on-grade.</t>
         </is>
@@ -1653,7 +1453,7 @@
           <t>Foundations &amp; anchoring</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Hurricane tie-downs / engineered anchoring to slab</t>
         </is>
@@ -1673,31 +1473,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G12" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H12" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="I12" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="J12" s="4" t="n">
         <v>54000</v>
       </c>
-      <c r="K12" s="5" t="n">
+      <c r="K12" s="4" t="n">
         <v>81000</v>
       </c>
-      <c r="L12" s="5" t="n">
+      <c r="L12" s="4" t="n">
         <v>45000</v>
       </c>
-      <c r="M12" s="5" t="n">
+      <c r="M12" s="4" t="n">
         <v>180000</v>
       </c>
-      <c r="N12" s="5" t="n">
+      <c r="N12" s="4" t="n">
         <v>180000</v>
       </c>
-      <c r="O12" s="7" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>Belize hurricane corridor. Confirm factory wind package separately.</t>
         </is>
@@ -1714,7 +1514,7 @@
           <t>Foundations &amp; anchoring</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Crane campaign — set container unit</t>
         </is>
@@ -1734,60 +1534,60 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="4" t="n">
         <v>800</v>
       </c>
-      <c r="H13" s="5" t="n">
+      <c r="H13" s="4" t="n">
         <v>800</v>
       </c>
-      <c r="I13" s="5" t="n">
+      <c r="I13" s="4" t="n">
         <v>800</v>
       </c>
-      <c r="J13" s="5" t="n">
+      <c r="J13" s="4" t="n">
         <v>24000</v>
       </c>
-      <c r="K13" s="5" t="n">
+      <c r="K13" s="4" t="n">
         <v>36000</v>
       </c>
-      <c r="L13" s="5" t="n">
+      <c r="L13" s="4" t="n">
         <v>20000</v>
       </c>
-      <c r="M13" s="5" t="n">
+      <c r="M13" s="4" t="n">
         <v>80000</v>
       </c>
-      <c r="N13" s="5" t="n">
+      <c r="N13" s="4" t="n">
         <v>80000</v>
       </c>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>Shared crawler plant hire only. Crew to assemble the module on the pad is 11.01 — supplier hours at US$28/hr. Mix 80% Belizean / 20% China tech.</t>
+      <c r="O13" s="5" t="inlineStr">
+        <is>
+          <t>Shared crawler plant hire only. Crew to assemble the module on the pad is Div 11.01 — US$28/hr. Mix 80% Belizean / 20% China tech.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Split air &amp; solar PV — no battery</t>
         </is>
       </c>
-      <c r="C14" s="13" t="n"/>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="13" t="n"/>
-      <c r="H14" s="13" t="n"/>
-      <c r="I14" s="13" t="n"/>
-      <c r="J14" s="13" t="n"/>
-      <c r="K14" s="13" t="n"/>
-      <c r="L14" s="13" t="n"/>
-      <c r="M14" s="13" t="n"/>
-      <c r="N14" s="13" t="n"/>
-      <c r="O14" s="13" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
+      <c r="H14" s="10" t="n"/>
+      <c r="I14" s="10" t="n"/>
+      <c r="J14" s="10" t="n"/>
+      <c r="K14" s="10" t="n"/>
+      <c r="L14" s="10" t="n"/>
+      <c r="M14" s="10" t="n"/>
+      <c r="N14" s="10" t="n"/>
+      <c r="O14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1800,7 +1600,7 @@
           <t>Split air &amp; solar PV — no battery</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Split-system air conditioner, installed</t>
         </is>
@@ -1820,31 +1620,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="4" t="n">
         <v>1200</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H15" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="I15" s="5" t="n">
+      <c r="I15" s="4" t="n">
         <v>2400</v>
       </c>
-      <c r="J15" s="5" t="n">
+      <c r="J15" s="4" t="n">
         <v>36000</v>
       </c>
-      <c r="K15" s="5" t="n">
+      <c r="K15" s="4" t="n">
         <v>81000</v>
       </c>
-      <c r="L15" s="5" t="n">
+      <c r="L15" s="4" t="n">
         <v>60000</v>
       </c>
-      <c r="M15" s="5" t="n">
+      <c r="M15" s="4" t="n">
         <v>177000</v>
       </c>
-      <c r="N15" s="5" t="n">
+      <c r="N15" s="4" t="n">
         <v>177000</v>
       </c>
-      <c r="O15" s="7" t="inlineStr">
+      <c r="O15" s="5" t="inlineStr">
         <is>
           <t>12k / 18k / 24k BTU. In house MEP — not in Homes only (FOB China). Not in the standard module fittings.</t>
         </is>
@@ -1861,7 +1661,7 @@
           <t>Split air &amp; solar PV — no battery</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Rooftop solar PV modules (panels only — equipment)</t>
         </is>
@@ -1881,31 +1681,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="G16" s="4" t="n">
         <v>2550</v>
       </c>
-      <c r="H16" s="5" t="n">
+      <c r="H16" s="4" t="n">
         <v>3400</v>
       </c>
-      <c r="I16" s="5" t="n">
+      <c r="I16" s="4" t="n">
         <v>4250</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="J16" s="4" t="n">
         <v>76500</v>
       </c>
-      <c r="K16" s="5" t="n">
+      <c r="K16" s="4" t="n">
         <v>153000</v>
       </c>
-      <c r="L16" s="5" t="n">
+      <c r="L16" s="4" t="n">
         <v>106250</v>
       </c>
-      <c r="M16" s="5" t="n">
+      <c r="M16" s="4" t="n">
         <v>335750</v>
       </c>
-      <c r="N16" s="5" t="n">
+      <c r="N16" s="4" t="n">
         <v>335750</v>
       </c>
-      <c r="O16" s="7" t="inlineStr">
+      <c r="O16" s="5" t="inlineStr">
         <is>
           <t>8 / 10 / 13 × 400 W modules = 3.2 / 4.0 / 5.2 kW array. Equipment only — no install labour. Install is 11.02 at $19.40/hr EST. (70% Belizean electrician / 30% China PV tech).</t>
         </is>
@@ -1922,7 +1722,7 @@
           <t>Split air &amp; solar PV — no battery</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Hybrid inverter, grid-tie — no battery (equipment)</t>
         </is>
@@ -1942,31 +1742,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n">
+      <c r="G17" s="4" t="n">
         <v>1650</v>
       </c>
-      <c r="H17" s="5" t="n">
+      <c r="H17" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="I17" s="5" t="n">
+      <c r="I17" s="4" t="n">
         <v>1950</v>
       </c>
-      <c r="J17" s="5" t="n">
+      <c r="J17" s="4" t="n">
         <v>49500</v>
       </c>
-      <c r="K17" s="5" t="n">
+      <c r="K17" s="4" t="n">
         <v>81000</v>
       </c>
-      <c r="L17" s="5" t="n">
+      <c r="L17" s="4" t="n">
         <v>48750</v>
       </c>
-      <c r="M17" s="5" t="n">
+      <c r="M17" s="4" t="n">
         <v>179250</v>
       </c>
-      <c r="N17" s="5" t="n">
+      <c r="N17" s="4" t="n">
         <v>179250</v>
       </c>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="O17" s="5" t="inlineStr">
         <is>
           <t>3 / 4 / 5 kW hybrid inverter, grid-interactive. Equipment only — no install labour. No battery. Install is 11.02 at $19.40/hr EST.</t>
         </is>
@@ -1983,7 +1783,7 @@
           <t>Split air &amp; solar PV — no battery</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>PV mounting hardware — rails, clamps, bonding kit (materials only)</t>
         </is>
@@ -2003,286 +1803,286 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="G18" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H18" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="I18" s="5" t="n">
+      <c r="I18" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="J18" s="4" t="n">
         <v>9000</v>
       </c>
-      <c r="K18" s="5" t="n">
+      <c r="K18" s="4" t="n">
         <v>13500</v>
       </c>
-      <c r="L18" s="5" t="n">
+      <c r="L18" s="4" t="n">
         <v>7500</v>
       </c>
-      <c r="M18" s="5" t="n">
+      <c r="M18" s="4" t="n">
         <v>30000</v>
       </c>
-      <c r="N18" s="5" t="n">
+      <c r="N18" s="4" t="n">
         <v>30000</v>
       </c>
-      <c r="O18" s="7" t="inlineStr">
+      <c r="O18" s="5" t="inlineStr">
         <is>
           <t>Materials only. Roof install labour is 11.02 at $19.40/hr EST. (70% Belizean / 30% China) — not in this $300.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>04.05</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Split air &amp; solar PV — no battery</t>
         </is>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>Battery energy storage (LiFePO4) — NOT INCLUDED</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>EXCL. · TBD</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="G19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="G19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N19" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="O19" s="14" t="inlineStr">
+      <c r="O19" s="12" t="inlineStr">
         <is>
           <t>No battery storage is included with the PV arrays. Grid-tie only. Optional later upgrade — rate left blank until the Government elects storage.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Electrical — village</t>
         </is>
       </c>
-      <c r="C20" s="13" t="n"/>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
-      <c r="J20" s="13" t="n"/>
-      <c r="K20" s="13" t="n"/>
-      <c r="L20" s="13" t="n"/>
-      <c r="M20" s="13" t="n"/>
-      <c r="N20" s="13" t="n"/>
-      <c r="O20" s="13" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
+      <c r="H20" s="10" t="n"/>
+      <c r="I20" s="10" t="n"/>
+      <c r="J20" s="10" t="n"/>
+      <c r="K20" s="10" t="n"/>
+      <c r="L20" s="10" t="n"/>
+      <c r="M20" s="10" t="n"/>
+      <c r="N20" s="10" t="n"/>
+      <c r="O20" s="10" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>05.01</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>Electrical — village</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>Padmount transformers — 2 × 500 kVA, 11–13.2 kV / 400Y/230V</t>
         </is>
       </c>
-      <c r="D21" s="17" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>nr</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F21" s="17" t="inlineStr">
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G21" s="19" t="n">
+      <c r="G21" s="17" t="n">
         <v>48000</v>
       </c>
-      <c r="H21" s="19" t="n">
+      <c r="H21" s="17" t="n">
         <v>48000</v>
       </c>
-      <c r="I21" s="19" t="n">
+      <c r="I21" s="17" t="n">
         <v>48000</v>
       </c>
-      <c r="J21" s="17" t="n"/>
-      <c r="K21" s="17" t="n"/>
-      <c r="L21" s="17" t="n"/>
-      <c r="M21" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="19" t="n">
+      <c r="J21" s="15" t="n"/>
+      <c r="K21" s="15" t="n"/>
+      <c r="L21" s="15" t="n"/>
+      <c r="M21" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="17" t="n">
         <v>96000</v>
       </c>
-      <c r="O21" s="18" t="inlineStr">
+      <c r="O21" s="16" t="inlineStr">
         <is>
           <t>Scaled from RTOAC Div (o) dry-type / utility transformer logic. Village, not civic 1500 kVA.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>05.02</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>Electrical — village</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>MV/LV distribution, laterals, service entrance, 100 meters</t>
         </is>
       </c>
-      <c r="D22" s="17" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F22" s="17" t="inlineStr">
+      <c r="F22" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G22" s="19" t="n">
+      <c r="G22" s="17" t="n">
         <v>520000</v>
       </c>
-      <c r="H22" s="19" t="n">
+      <c r="H22" s="17" t="n">
         <v>520000</v>
       </c>
-      <c r="I22" s="19" t="n">
+      <c r="I22" s="17" t="n">
         <v>520000</v>
       </c>
-      <c r="J22" s="17" t="n"/>
-      <c r="K22" s="17" t="n"/>
-      <c r="L22" s="17" t="n"/>
-      <c r="M22" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="19" t="n">
+      <c r="J22" s="15" t="n"/>
+      <c r="K22" s="15" t="n"/>
+      <c r="L22" s="15" t="n"/>
+      <c r="M22" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="17" t="n">
         <v>520000</v>
       </c>
-      <c r="O22" s="18" t="inlineStr">
+      <c r="O22" s="16" t="inlineStr">
         <is>
           <t>RTOAC Div (o) feeders + branch, scaled to 100 dwellings.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>05.03</t>
         </is>
       </c>
-      <c r="B23" s="17" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t>Electrical — village</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>Street lighting — LED, 80 nr along avenues</t>
         </is>
       </c>
-      <c r="D23" s="17" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>nr</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E23" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F23" s="17" t="inlineStr">
+      <c r="F23" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G23" s="19" t="n">
+      <c r="G23" s="17" t="n">
         <v>1200</v>
       </c>
-      <c r="H23" s="19" t="n">
+      <c r="H23" s="17" t="n">
         <v>1200</v>
       </c>
-      <c r="I23" s="19" t="n">
+      <c r="I23" s="17" t="n">
         <v>1200</v>
       </c>
-      <c r="J23" s="17" t="n"/>
-      <c r="K23" s="17" t="n"/>
-      <c r="L23" s="17" t="n"/>
-      <c r="M23" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="19" t="n">
+      <c r="J23" s="15" t="n"/>
+      <c r="K23" s="15" t="n"/>
+      <c r="L23" s="15" t="n"/>
+      <c r="M23" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="17" t="n">
         <v>96000</v>
       </c>
-      <c r="O23" s="18" t="inlineStr">
+      <c r="O23" s="16" t="inlineStr">
         <is>
           <t>80 columns. Qty carried in projectQty via lumpQty.</t>
         </is>
@@ -2299,7 +2099,7 @@
           <t>Electrical — village</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>House consumer unit, branch wiring allowance (beyond factory)</t>
         </is>
@@ -2319,170 +2119,170 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="G24" s="4" t="n">
         <v>850</v>
       </c>
-      <c r="H24" s="5" t="n">
+      <c r="H24" s="4" t="n">
         <v>1150</v>
       </c>
-      <c r="I24" s="5" t="n">
+      <c r="I24" s="4" t="n">
         <v>1250</v>
       </c>
-      <c r="J24" s="5" t="n">
+      <c r="J24" s="4" t="n">
         <v>25500</v>
       </c>
-      <c r="K24" s="5" t="n">
+      <c r="K24" s="4" t="n">
         <v>51750</v>
       </c>
-      <c r="L24" s="5" t="n">
+      <c r="L24" s="4" t="n">
         <v>31250</v>
       </c>
-      <c r="M24" s="5" t="n">
+      <c r="M24" s="4" t="n">
         <v>108500</v>
       </c>
-      <c r="N24" s="5" t="n">
+      <c r="N24" s="4" t="n">
         <v>108500</v>
       </c>
-      <c r="O24" s="7" t="inlineStr">
+      <c r="O24" s="5" t="inlineStr">
         <is>
           <t>Factory ships a fitted board; this is site hookup and extra devices.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>05.05</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Electrical — village</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>Civic pavilion + gatehouse electrical</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E25" s="17" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F25" s="17" t="inlineStr">
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G25" s="19" t="n">
+      <c r="G25" s="17" t="n">
         <v>42000</v>
       </c>
-      <c r="H25" s="19" t="n">
+      <c r="H25" s="17" t="n">
         <v>42000</v>
       </c>
-      <c r="I25" s="19" t="n">
+      <c r="I25" s="17" t="n">
         <v>42000</v>
       </c>
-      <c r="J25" s="17" t="n"/>
-      <c r="K25" s="17" t="n"/>
-      <c r="L25" s="17" t="n"/>
-      <c r="M25" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="19" t="n">
+      <c r="J25" s="15" t="n"/>
+      <c r="K25" s="15" t="n"/>
+      <c r="L25" s="15" t="n"/>
+      <c r="M25" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="17" t="n">
         <v>42000</v>
       </c>
-      <c r="O25" s="18" t="inlineStr">
+      <c r="O25" s="16" t="inlineStr">
         <is>
           <t>RTOAC-inspired builders-work electrical, civic scale.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="17" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>05.06</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Electrical — village</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>Testing, commissioning, as-builts, coordination study</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr">
+      <c r="E26" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F26" s="17" t="inlineStr">
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G26" s="19" t="n">
+      <c r="G26" s="17" t="n">
         <v>55000</v>
       </c>
-      <c r="H26" s="19" t="n">
+      <c r="H26" s="17" t="n">
         <v>55000</v>
       </c>
-      <c r="I26" s="19" t="n">
+      <c r="I26" s="17" t="n">
         <v>55000</v>
       </c>
-      <c r="J26" s="17" t="n"/>
-      <c r="K26" s="17" t="n"/>
-      <c r="L26" s="17" t="n"/>
-      <c r="M26" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="19" t="n">
+      <c r="J26" s="15" t="n"/>
+      <c r="K26" s="15" t="n"/>
+      <c r="L26" s="15" t="n"/>
+      <c r="M26" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="17" t="n">
         <v>55000</v>
       </c>
-      <c r="O26" s="18" t="inlineStr">
+      <c r="O26" s="16" t="inlineStr">
         <is>
           <t>RTOAC Div (o) testing &amp; closeout, scaled.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Plumbing &amp; sanitary</t>
         </is>
       </c>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
-      <c r="G27" s="13" t="n"/>
-      <c r="H27" s="13" t="n"/>
-      <c r="I27" s="13" t="n"/>
-      <c r="J27" s="13" t="n"/>
-      <c r="K27" s="13" t="n"/>
-      <c r="L27" s="13" t="n"/>
-      <c r="M27" s="13" t="n"/>
-      <c r="N27" s="13" t="n"/>
-      <c r="O27" s="13" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="10" t="n"/>
+      <c r="J27" s="10" t="n"/>
+      <c r="K27" s="10" t="n"/>
+      <c r="L27" s="10" t="n"/>
+      <c r="M27" s="10" t="n"/>
+      <c r="N27" s="10" t="n"/>
+      <c r="O27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2495,7 +2295,7 @@
           <t>Plumbing &amp; sanitary</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Sanitaryware — toilet, shower, kitchen sink (in the module)</t>
         </is>
@@ -2515,86 +2315,86 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G28" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="7" t="inlineStr">
+      <c r="G28" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="5" t="inlineStr">
         <is>
           <t>INCL. in the basic shell — $0 extra. Toilet, shower cube, wash-basin, kitchen sink and cabinet ship in the box. Split air is 04.01. Range/fridge is 08.01.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>06.02</t>
         </is>
       </c>
-      <c r="B29" s="17" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Plumbing &amp; sanitary</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>Village potable water — elevated tank, mains to 100 lots, disinfection</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E29" s="17" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F29" s="17" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G29" s="19" t="n">
+      <c r="G29" s="17" t="n">
         <v>410000</v>
       </c>
-      <c r="H29" s="19" t="n">
+      <c r="H29" s="17" t="n">
         <v>410000</v>
       </c>
-      <c r="I29" s="19" t="n">
+      <c r="I29" s="17" t="n">
         <v>410000</v>
       </c>
-      <c r="J29" s="17" t="n"/>
-      <c r="K29" s="17" t="n"/>
-      <c r="L29" s="17" t="n"/>
-      <c r="M29" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N29" s="19" t="n">
+      <c r="J29" s="15" t="n"/>
+      <c r="K29" s="15" t="n"/>
+      <c r="L29" s="15" t="n"/>
+      <c r="M29" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="17" t="n">
         <v>410000</v>
       </c>
-      <c r="O29" s="18" t="inlineStr">
+      <c r="O29" s="16" t="inlineStr">
         <is>
           <t>RTOAC plumbing distribution analog — drinking-water loop for 100 lots. Not in Homes only. WWTP (sewage) is 06.04, separate.</t>
         </is>
@@ -2611,7 +2411,7 @@
           <t>Plumbing &amp; sanitary</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>House water lateral + yard cistern stub</t>
         </is>
@@ -2631,86 +2431,86 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="G30" s="4" t="n">
         <v>1150</v>
       </c>
-      <c r="H30" s="5" t="n">
+      <c r="H30" s="4" t="n">
         <v>1150</v>
       </c>
-      <c r="I30" s="5" t="n">
+      <c r="I30" s="4" t="n">
         <v>1150</v>
       </c>
-      <c r="J30" s="5" t="n">
+      <c r="J30" s="4" t="n">
         <v>34500</v>
       </c>
-      <c r="K30" s="5" t="n">
+      <c r="K30" s="4" t="n">
         <v>51750</v>
       </c>
-      <c r="L30" s="5" t="n">
+      <c r="L30" s="4" t="n">
         <v>28750</v>
       </c>
-      <c r="M30" s="5" t="n">
+      <c r="M30" s="4" t="n">
         <v>115000</v>
       </c>
-      <c r="N30" s="5" t="n">
+      <c r="N30" s="4" t="n">
         <v>115000</v>
       </c>
-      <c r="O30" s="7" t="inlineStr">
+      <c r="O30" s="5" t="inlineStr">
         <is>
           <t>Single connection point per pad.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="17" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>06.04</t>
         </is>
       </c>
-      <c r="B31" s="17" t="inlineStr">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>Plumbing &amp; sanitary</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>WWTP — wastewater treatment plant (shared sewage plant for 100 lots)</t>
         </is>
       </c>
-      <c r="D31" s="17" t="inlineStr">
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E31" s="17" t="inlineStr">
+      <c r="E31" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F31" s="17" t="inlineStr">
+      <c r="F31" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G31" s="19" t="n">
+      <c r="G31" s="17" t="n">
         <v>380000</v>
       </c>
-      <c r="H31" s="19" t="n">
+      <c r="H31" s="17" t="n">
         <v>380000</v>
       </c>
-      <c r="I31" s="19" t="n">
+      <c r="I31" s="17" t="n">
         <v>380000</v>
       </c>
-      <c r="J31" s="17" t="n"/>
-      <c r="K31" s="17" t="n"/>
-      <c r="L31" s="17" t="n"/>
-      <c r="M31" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N31" s="19" t="n">
+      <c r="J31" s="15" t="n"/>
+      <c r="K31" s="15" t="n"/>
+      <c r="L31" s="15" t="n"/>
+      <c r="M31" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="17" t="n">
         <v>380000</v>
       </c>
-      <c r="O31" s="18" t="inlineStr">
+      <c r="O31" s="16" t="inlineStr">
         <is>
           <t>WWTP = wastewater treatment plant. One shared sewage plant instead of 100 septic tanks. Not in Homes only. Not part of Civic extras (gate/plaza/trees).</t>
         </is>
@@ -2727,7 +2527,7 @@
           <t>Plumbing &amp; sanitary</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Sewer laterals — pad to collector</t>
         </is>
@@ -2747,56 +2547,56 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="G32" s="4" t="n">
         <v>980</v>
       </c>
-      <c r="H32" s="5" t="n">
+      <c r="H32" s="4" t="n">
         <v>980</v>
       </c>
-      <c r="I32" s="5" t="n">
+      <c r="I32" s="4" t="n">
         <v>980</v>
       </c>
-      <c r="J32" s="5" t="n">
+      <c r="J32" s="4" t="n">
         <v>29400</v>
       </c>
-      <c r="K32" s="5" t="n">
+      <c r="K32" s="4" t="n">
         <v>44100</v>
       </c>
-      <c r="L32" s="5" t="n">
+      <c r="L32" s="4" t="n">
         <v>24500</v>
       </c>
-      <c r="M32" s="5" t="n">
+      <c r="M32" s="4" t="n">
         <v>98000</v>
       </c>
-      <c r="N32" s="5" t="n">
+      <c r="N32" s="4" t="n">
         <v>98000</v>
       </c>
-      <c r="O32" s="7" t="inlineStr"/>
+      <c r="O32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Interior finishes</t>
         </is>
       </c>
-      <c r="C33" s="13" t="n"/>
-      <c r="D33" s="13" t="n"/>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n"/>
-      <c r="G33" s="13" t="n"/>
-      <c r="H33" s="13" t="n"/>
-      <c r="I33" s="13" t="n"/>
-      <c r="J33" s="13" t="n"/>
-      <c r="K33" s="13" t="n"/>
-      <c r="L33" s="13" t="n"/>
-      <c r="M33" s="13" t="n"/>
-      <c r="N33" s="13" t="n"/>
-      <c r="O33" s="13" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="10" t="n"/>
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="10" t="n"/>
+      <c r="H33" s="10" t="n"/>
+      <c r="I33" s="10" t="n"/>
+      <c r="J33" s="10" t="n"/>
+      <c r="K33" s="10" t="n"/>
+      <c r="L33" s="10" t="n"/>
+      <c r="M33" s="10" t="n"/>
+      <c r="N33" s="10" t="n"/>
+      <c r="O33" s="10" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2809,7 +2609,7 @@
           <t>Interior finishes</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Floor finishes — government spec (vinyl / sealed)</t>
         </is>
@@ -2829,31 +2629,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G34" s="5" t="n">
+      <c r="G34" s="4" t="n">
         <v>1250</v>
       </c>
-      <c r="H34" s="5" t="n">
+      <c r="H34" s="4" t="n">
         <v>2200</v>
       </c>
-      <c r="I34" s="5" t="n">
+      <c r="I34" s="4" t="n">
         <v>2200</v>
       </c>
-      <c r="J34" s="5" t="n">
+      <c r="J34" s="4" t="n">
         <v>37500</v>
       </c>
-      <c r="K34" s="5" t="n">
+      <c r="K34" s="4" t="n">
         <v>99000</v>
       </c>
-      <c r="L34" s="5" t="n">
+      <c r="L34" s="4" t="n">
         <v>55000</v>
       </c>
-      <c r="M34" s="5" t="n">
+      <c r="M34" s="4" t="n">
         <v>191500</v>
       </c>
-      <c r="N34" s="5" t="n">
+      <c r="N34" s="4" t="n">
         <v>191500</v>
       </c>
-      <c r="O34" s="7" t="inlineStr">
+      <c r="O34" s="5" t="inlineStr">
         <is>
           <t>RTOAC Div (f) analog at housing spec, not Porcelanosa stone.</t>
         </is>
@@ -2870,7 +2670,7 @@
           <t>Interior finishes</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>Wall finishes / paint</t>
         </is>
@@ -2890,31 +2690,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G35" s="4" t="n">
         <v>620</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H35" s="4" t="n">
         <v>980</v>
       </c>
-      <c r="I35" s="5" t="n">
+      <c r="I35" s="4" t="n">
         <v>1050</v>
       </c>
-      <c r="J35" s="5" t="n">
+      <c r="J35" s="4" t="n">
         <v>18600</v>
       </c>
-      <c r="K35" s="5" t="n">
+      <c r="K35" s="4" t="n">
         <v>44100</v>
       </c>
-      <c r="L35" s="5" t="n">
+      <c r="L35" s="4" t="n">
         <v>26250</v>
       </c>
-      <c r="M35" s="5" t="n">
+      <c r="M35" s="4" t="n">
         <v>88950</v>
       </c>
-      <c r="N35" s="5" t="n">
+      <c r="N35" s="4" t="n">
         <v>88950</v>
       </c>
-      <c r="O35" s="7" t="inlineStr">
+      <c r="O35" s="5" t="inlineStr">
         <is>
           <t>RTOAC paint rates, housing area.</t>
         </is>
@@ -2931,7 +2731,7 @@
           <t>Interior finishes</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>Ceilings — factory + make-good</t>
         </is>
@@ -2951,31 +2751,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G36" s="5" t="n">
+      <c r="G36" s="4" t="n">
         <v>280</v>
       </c>
-      <c r="H36" s="5" t="n">
+      <c r="H36" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="I36" s="5" t="n">
+      <c r="I36" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="J36" s="5" t="n">
+      <c r="J36" s="4" t="n">
         <v>8400</v>
       </c>
-      <c r="K36" s="5" t="n">
+      <c r="K36" s="4" t="n">
         <v>18900</v>
       </c>
-      <c r="L36" s="5" t="n">
+      <c r="L36" s="4" t="n">
         <v>10500</v>
       </c>
-      <c r="M36" s="5" t="n">
+      <c r="M36" s="4" t="n">
         <v>37800</v>
       </c>
-      <c r="N36" s="5" t="n">
+      <c r="N36" s="4" t="n">
         <v>37800</v>
       </c>
-      <c r="O36" s="7" t="inlineStr">
+      <c r="O36" s="5" t="inlineStr">
         <is>
           <t>RTOAC Div (e) analog.</t>
         </is>
@@ -2992,7 +2792,7 @@
           <t>Interior finishes</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>Internal doors — factory sets</t>
         </is>
@@ -3012,31 +2812,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G37" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N37" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O37" s="7" t="inlineStr">
+      <c r="G37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O37" s="5" t="inlineStr">
         <is>
           <t>In 01.01. RTOAC Div (h) analog already in the module.</t>
         </is>
@@ -3053,7 +2853,7 @@
           <t>Interior finishes</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>Kitchen millwork make-good (factory + local)</t>
         </is>
@@ -3073,31 +2873,31 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G38" s="5" t="n">
+      <c r="G38" s="4" t="n">
         <v>350</v>
       </c>
-      <c r="H38" s="5" t="n">
+      <c r="H38" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="I38" s="5" t="n">
+      <c r="I38" s="4" t="n">
         <v>520</v>
       </c>
-      <c r="J38" s="5" t="n">
+      <c r="J38" s="4" t="n">
         <v>10500</v>
       </c>
-      <c r="K38" s="5" t="n">
+      <c r="K38" s="4" t="n">
         <v>21600</v>
       </c>
-      <c r="L38" s="5" t="n">
+      <c r="L38" s="4" t="n">
         <v>13000</v>
       </c>
-      <c r="M38" s="5" t="n">
+      <c r="M38" s="4" t="n">
         <v>45100</v>
       </c>
-      <c r="N38" s="5" t="n">
+      <c r="N38" s="4" t="n">
         <v>45100</v>
       </c>
-      <c r="O38" s="7" t="inlineStr">
+      <c r="O38" s="5" t="inlineStr">
         <is>
           <t>RTOAC Div (i) analog — kitchen cabinet already in the module.</t>
         </is>
@@ -3114,7 +2914,7 @@
           <t>Interior finishes</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>Light fixtures — LED house allowance</t>
         </is>
@@ -3134,60 +2934,60 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G39" s="5" t="n">
+      <c r="G39" s="4" t="n">
         <v>650</v>
       </c>
-      <c r="H39" s="5" t="n">
+      <c r="H39" s="4" t="n">
         <v>1100</v>
       </c>
-      <c r="I39" s="5" t="n">
+      <c r="I39" s="4" t="n">
         <v>1250</v>
       </c>
-      <c r="J39" s="5" t="n">
+      <c r="J39" s="4" t="n">
         <v>19500</v>
       </c>
-      <c r="K39" s="5" t="n">
+      <c r="K39" s="4" t="n">
         <v>49500</v>
       </c>
-      <c r="L39" s="5" t="n">
+      <c r="L39" s="4" t="n">
         <v>31250</v>
       </c>
-      <c r="M39" s="5" t="n">
+      <c r="M39" s="4" t="n">
         <v>100250</v>
       </c>
-      <c r="N39" s="5" t="n">
+      <c r="N39" s="4" t="n">
         <v>100250</v>
       </c>
-      <c r="O39" s="7" t="inlineStr">
+      <c r="O39" s="5" t="inlineStr">
         <is>
           <t>RTOAC Div (g) analog at housing count.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>08</t>
         </is>
       </c>
-      <c r="B40" s="13" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="C40" s="13" t="n"/>
-      <c r="D40" s="13" t="n"/>
-      <c r="E40" s="13" t="n"/>
-      <c r="F40" s="13" t="n"/>
-      <c r="G40" s="13" t="n"/>
-      <c r="H40" s="13" t="n"/>
-      <c r="I40" s="13" t="n"/>
-      <c r="J40" s="13" t="n"/>
-      <c r="K40" s="13" t="n"/>
-      <c r="L40" s="13" t="n"/>
-      <c r="M40" s="13" t="n"/>
-      <c r="N40" s="13" t="n"/>
-      <c r="O40" s="13" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="10" t="n"/>
+      <c r="H40" s="10" t="n"/>
+      <c r="I40" s="10" t="n"/>
+      <c r="J40" s="10" t="n"/>
+      <c r="K40" s="10" t="n"/>
+      <c r="L40" s="10" t="n"/>
+      <c r="M40" s="10" t="n"/>
+      <c r="N40" s="10" t="n"/>
+      <c r="O40" s="10" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3200,7 +3000,7 @@
           <t>Appliances</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr">
         <is>
           <t>Range / cooktop + refrigerator package</t>
         </is>
@@ -3220,60 +3020,60 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G41" s="5" t="n">
+      <c r="G41" s="4" t="n">
         <v>1400</v>
       </c>
-      <c r="H41" s="5" t="n">
+      <c r="H41" s="4" t="n">
         <v>1800</v>
       </c>
-      <c r="I41" s="5" t="n">
+      <c r="I41" s="4" t="n">
         <v>2100</v>
       </c>
-      <c r="J41" s="5" t="n">
+      <c r="J41" s="4" t="n">
         <v>42000</v>
       </c>
-      <c r="K41" s="5" t="n">
+      <c r="K41" s="4" t="n">
         <v>81000</v>
       </c>
-      <c r="L41" s="5" t="n">
+      <c r="L41" s="4" t="n">
         <v>52500</v>
       </c>
-      <c r="M41" s="5" t="n">
+      <c r="M41" s="4" t="n">
         <v>175500</v>
       </c>
-      <c r="N41" s="5" t="n">
+      <c r="N41" s="4" t="n">
         <v>175500</v>
       </c>
-      <c r="O41" s="7" t="inlineStr">
+      <c r="O41" s="5" t="inlineStr">
         <is>
           <t>Not in the basic shell. Gas stove is optional at the supplier and is not in this price. Washer/dryer not in base.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B42" s="13" t="inlineStr">
+      <c r="B42" s="10" t="inlineStr">
         <is>
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C42" s="13" t="n"/>
-      <c r="D42" s="13" t="n"/>
-      <c r="E42" s="13" t="n"/>
-      <c r="F42" s="13" t="n"/>
-      <c r="G42" s="13" t="n"/>
-      <c r="H42" s="13" t="n"/>
-      <c r="I42" s="13" t="n"/>
-      <c r="J42" s="13" t="n"/>
-      <c r="K42" s="13" t="n"/>
-      <c r="L42" s="13" t="n"/>
-      <c r="M42" s="13" t="n"/>
-      <c r="N42" s="13" t="n"/>
-      <c r="O42" s="13" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="10" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="10" t="n"/>
+      <c r="I42" s="10" t="n"/>
+      <c r="J42" s="10" t="n"/>
+      <c r="K42" s="10" t="n"/>
+      <c r="L42" s="10" t="n"/>
+      <c r="M42" s="10" t="n"/>
+      <c r="N42" s="10" t="n"/>
+      <c r="O42" s="10" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3286,7 +3086,7 @@
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>Site clearing, stripping, enabling (~33 acres)</t>
         </is>
@@ -3306,77 +3106,77 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G43" s="5" t="n">
+      <c r="G43" s="4" t="n">
         <v>185000</v>
       </c>
-      <c r="H43" s="5" t="n">
+      <c r="H43" s="4" t="n">
         <v>185000</v>
       </c>
-      <c r="I43" s="5" t="n">
+      <c r="I43" s="4" t="n">
         <v>185000</v>
       </c>
-      <c r="M43" s="5" t="n">
+      <c r="M43" s="4" t="n">
         <v>185000</v>
       </c>
-      <c r="N43" s="5" t="n">
+      <c r="N43" s="4" t="n">
         <v>185000</v>
       </c>
-      <c r="O43" s="7" t="inlineStr">
+      <c r="O43" s="5" t="inlineStr">
         <is>
           <t>RTOAC Div (a) demolition analog — greenfield enabling.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>09.02</t>
         </is>
       </c>
-      <c r="B44" s="17" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C44" s="16" t="inlineStr">
         <is>
           <t>Village roads — gravel avenues, lot access, drainage swales</t>
         </is>
       </c>
-      <c r="D44" s="17" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E44" s="17" t="inlineStr">
+      <c r="E44" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F44" s="17" t="inlineStr">
+      <c r="F44" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G44" s="19" t="n">
+      <c r="G44" s="17" t="n">
         <v>620000</v>
       </c>
-      <c r="H44" s="19" t="n">
+      <c r="H44" s="17" t="n">
         <v>620000</v>
       </c>
-      <c r="I44" s="19" t="n">
+      <c r="I44" s="17" t="n">
         <v>620000</v>
       </c>
-      <c r="J44" s="17" t="n"/>
-      <c r="K44" s="17" t="n"/>
-      <c r="L44" s="17" t="n"/>
-      <c r="M44" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N44" s="19" t="n">
+      <c r="J44" s="15" t="n"/>
+      <c r="K44" s="15" t="n"/>
+      <c r="L44" s="15" t="n"/>
+      <c r="M44" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="17" t="n">
         <v>620000</v>
       </c>
-      <c r="O44" s="18" t="inlineStr">
+      <c r="O44" s="16" t="inlineStr">
         <is>
           <t>RTOAC Div (m) external works analog. Gravel, not asphalt. Not in Homes only. Civic extras (gate/plaza) are 09.04–09.06.</t>
         </is>
@@ -3393,7 +3193,7 @@
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>Lot grading and pad preparation</t>
         </is>
@@ -3413,354 +3213,354 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="G45" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="H45" s="5" t="n">
+      <c r="H45" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="I45" s="5" t="n">
+      <c r="I45" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="J45" s="5" t="n">
+      <c r="J45" s="4" t="n">
         <v>12600</v>
       </c>
-      <c r="K45" s="5" t="n">
+      <c r="K45" s="4" t="n">
         <v>18900</v>
       </c>
-      <c r="L45" s="5" t="n">
+      <c r="L45" s="4" t="n">
         <v>10500</v>
       </c>
-      <c r="M45" s="5" t="n">
+      <c r="M45" s="4" t="n">
         <v>42000</v>
       </c>
-      <c r="N45" s="5" t="n">
+      <c r="N45" s="4" t="n">
         <v>42000</v>
       </c>
-      <c r="O45" s="7" t="inlineStr"/>
+      <c r="O45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>09.04</t>
         </is>
       </c>
-      <c r="B46" s="17" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C46" s="16" t="inlineStr">
         <is>
           <t>Perimeter fence + village gatehouse</t>
         </is>
       </c>
-      <c r="D46" s="17" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E46" s="17" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F46" s="17" t="inlineStr">
+      <c r="F46" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G46" s="19" t="n">
+      <c r="G46" s="17" t="n">
         <v>140000</v>
       </c>
-      <c r="H46" s="19" t="n">
+      <c r="H46" s="17" t="n">
         <v>140000</v>
       </c>
-      <c r="I46" s="19" t="n">
+      <c r="I46" s="17" t="n">
         <v>140000</v>
       </c>
-      <c r="J46" s="17" t="n"/>
-      <c r="K46" s="17" t="n"/>
-      <c r="L46" s="17" t="n"/>
-      <c r="M46" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N46" s="19" t="n">
+      <c r="J46" s="15" t="n"/>
+      <c r="K46" s="15" t="n"/>
+      <c r="L46" s="15" t="n"/>
+      <c r="M46" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N46" s="17" t="n">
         <v>140000</v>
       </c>
-      <c r="O46" s="18" t="inlineStr">
+      <c r="O46" s="16" t="inlineStr">
         <is>
           <t>RTOAC Div (l) security analog — gatehouse, not mantrap. Civic extra. Not roads, water, power, or WWTP.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="17" t="inlineStr">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>09.05</t>
         </is>
       </c>
-      <c r="B47" s="17" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
+      <c r="C47" s="16" t="inlineStr">
         <is>
           <t>Civic plaza + pavilion (community hall)</t>
         </is>
       </c>
-      <c r="D47" s="17" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E47" s="17" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F47" s="17" t="inlineStr">
+      <c r="F47" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G47" s="19" t="n">
+      <c r="G47" s="17" t="n">
         <v>185000</v>
       </c>
-      <c r="H47" s="19" t="n">
+      <c r="H47" s="17" t="n">
         <v>185000</v>
       </c>
-      <c r="I47" s="19" t="n">
+      <c r="I47" s="17" t="n">
         <v>185000</v>
       </c>
-      <c r="J47" s="17" t="n"/>
-      <c r="K47" s="17" t="n"/>
-      <c r="L47" s="17" t="n"/>
-      <c r="M47" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N47" s="19" t="n">
+      <c r="J47" s="15" t="n"/>
+      <c r="K47" s="15" t="n"/>
+      <c r="L47" s="15" t="n"/>
+      <c r="M47" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="17" t="n">
         <v>185000</v>
       </c>
-      <c r="O47" s="18" t="inlineStr">
+      <c r="O47" s="16" t="inlineStr">
         <is>
           <t>Open-air single-storey pavilion at the crossroads, gravel plaza, benches, civic green. Conceptual rendering on /civic. Not a two-storey hall. Civic extra — not village utilities.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="17" t="inlineStr">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>09.06</t>
         </is>
       </c>
-      <c r="B48" s="17" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C48" s="18" t="inlineStr">
+      <c r="C48" s="16" t="inlineStr">
         <is>
           <t>Street trees, lot grassing, civic green</t>
         </is>
       </c>
-      <c r="D48" s="17" t="inlineStr">
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E48" s="17" t="inlineStr">
+      <c r="E48" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F48" s="17" t="inlineStr">
+      <c r="F48" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G48" s="19" t="n">
+      <c r="G48" s="17" t="n">
         <v>95000</v>
       </c>
-      <c r="H48" s="19" t="n">
+      <c r="H48" s="17" t="n">
         <v>95000</v>
       </c>
-      <c r="I48" s="19" t="n">
+      <c r="I48" s="17" t="n">
         <v>95000</v>
       </c>
-      <c r="J48" s="17" t="n"/>
-      <c r="K48" s="17" t="n"/>
-      <c r="L48" s="17" t="n"/>
-      <c r="M48" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N48" s="19" t="n">
+      <c r="J48" s="15" t="n"/>
+      <c r="K48" s="15" t="n"/>
+      <c r="L48" s="15" t="n"/>
+      <c r="M48" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N48" s="17" t="n">
         <v>95000</v>
       </c>
-      <c r="O48" s="18" t="inlineStr"/>
+      <c r="O48" s="16" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="17" t="inlineStr">
+      <c r="A49" s="15" t="inlineStr">
         <is>
           <t>09.07</t>
         </is>
       </c>
-      <c r="B49" s="17" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>External works &amp; civic</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
+      <c r="C49" s="16" t="inlineStr">
         <is>
           <t>Stormwater — culverts, outfall, swale lining</t>
         </is>
       </c>
-      <c r="D49" s="17" t="inlineStr">
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>ls</t>
         </is>
       </c>
-      <c r="E49" s="17" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F49" s="17" t="inlineStr">
+      <c r="F49" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G49" s="19" t="n">
+      <c r="G49" s="17" t="n">
         <v>120000</v>
       </c>
-      <c r="H49" s="19" t="n">
+      <c r="H49" s="17" t="n">
         <v>120000</v>
       </c>
-      <c r="I49" s="19" t="n">
+      <c r="I49" s="17" t="n">
         <v>120000</v>
       </c>
-      <c r="J49" s="17" t="n"/>
-      <c r="K49" s="17" t="n"/>
-      <c r="L49" s="17" t="n"/>
-      <c r="M49" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N49" s="19" t="n">
+      <c r="J49" s="15" t="n"/>
+      <c r="K49" s="15" t="n"/>
+      <c r="L49" s="15" t="n"/>
+      <c r="M49" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N49" s="17" t="n">
         <v>120000</v>
       </c>
-      <c r="O49" s="18" t="inlineStr"/>
+      <c r="O49" s="16" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B50" s="13" t="inlineStr">
+      <c r="B50" s="10" t="inlineStr">
         <is>
           <t>FF&amp;E — furnished upgrade</t>
         </is>
       </c>
-      <c r="C50" s="13" t="n"/>
-      <c r="D50" s="13" t="n"/>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="13" t="n"/>
-      <c r="G50" s="13" t="n"/>
-      <c r="H50" s="13" t="n"/>
-      <c r="I50" s="13" t="n"/>
-      <c r="J50" s="13" t="n"/>
-      <c r="K50" s="13" t="n"/>
-      <c r="L50" s="13" t="n"/>
-      <c r="M50" s="13" t="n"/>
-      <c r="N50" s="13" t="n"/>
-      <c r="O50" s="13" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="10" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="10" t="n"/>
+      <c r="H50" s="10" t="n"/>
+      <c r="I50" s="10" t="n"/>
+      <c r="J50" s="10" t="n"/>
+      <c r="K50" s="10" t="n"/>
+      <c r="L50" s="10" t="n"/>
+      <c r="M50" s="10" t="n"/>
+      <c r="N50" s="10" t="n"/>
+      <c r="O50" s="10" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="17" t="inlineStr">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>10.01</t>
         </is>
       </c>
-      <c r="B51" s="17" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>FF&amp;E — furnished upgrade</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C51" s="16" t="inlineStr">
         <is>
           <t>Furniture / FF&amp;E package — beds, seating, dining, linens</t>
         </is>
       </c>
-      <c r="D51" s="17" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="E51" s="17" t="inlineStr">
+      <c r="E51" s="15" t="inlineStr">
         <is>
           <t>EST.</t>
         </is>
       </c>
-      <c r="F51" s="17" t="inlineStr">
+      <c r="F51" s="15" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G51" s="19" t="n">
+      <c r="G51" s="17" t="n">
         <v>3500</v>
       </c>
-      <c r="H51" s="19" t="n">
+      <c r="H51" s="17" t="n">
         <v>5500</v>
       </c>
-      <c r="I51" s="19" t="n">
+      <c r="I51" s="17" t="n">
         <v>7000</v>
       </c>
-      <c r="J51" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K51" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="L51" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M51" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N51" s="19" t="n">
+      <c r="J51" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N51" s="17" t="n">
         <v>527500</v>
       </c>
-      <c r="O51" s="18" t="inlineStr">
+      <c r="O51" s="16" t="inlineStr">
         <is>
           <t>Priced separately. Base proposal is unfurnished. Equal add to any style.</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B52" s="13" t="inlineStr">
+      <c r="B52" s="10" t="inlineStr">
         <is>
           <t>Labour &amp; duration</t>
         </is>
       </c>
-      <c r="C52" s="13" t="n"/>
-      <c r="D52" s="13" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
-      <c r="G52" s="13" t="n"/>
-      <c r="H52" s="13" t="n"/>
-      <c r="I52" s="13" t="n"/>
-      <c r="J52" s="13" t="n"/>
-      <c r="K52" s="13" t="n"/>
-      <c r="L52" s="13" t="n"/>
-      <c r="M52" s="13" t="n"/>
-      <c r="N52" s="13" t="n"/>
-      <c r="O52" s="13" t="n"/>
+      <c r="C52" s="10" t="n"/>
+      <c r="D52" s="10" t="n"/>
+      <c r="E52" s="10" t="n"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="10" t="n"/>
+      <c r="H52" s="10" t="n"/>
+      <c r="I52" s="10" t="n"/>
+      <c r="J52" s="10" t="n"/>
+      <c r="K52" s="10" t="n"/>
+      <c r="L52" s="10" t="n"/>
+      <c r="M52" s="10" t="n"/>
+      <c r="N52" s="10" t="n"/>
+      <c r="O52" s="10" t="n"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3773,7 +3573,7 @@
           <t>Labour &amp; duration</t>
         </is>
       </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="5" t="inlineStr">
         <is>
           <t>Module assembly on the pad (man-hours / home)</t>
         </is>
@@ -3793,155 +3593,155 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G53" s="20" t="n">
+      <c r="G53" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="H53" s="20" t="n">
+      <c r="H53" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="I53" s="20" t="n">
+      <c r="I53" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="J53" s="5" t="n">
+      <c r="J53" s="4" t="n">
         <v>35280</v>
       </c>
-      <c r="K53" s="5" t="n">
+      <c r="K53" s="4" t="n">
         <v>100800</v>
       </c>
-      <c r="L53" s="5" t="n">
+      <c r="L53" s="4" t="n">
         <v>56000</v>
       </c>
-      <c r="M53" s="5" t="n">
+      <c r="M53" s="4" t="n">
         <v>192080</v>
       </c>
-      <c r="N53" s="5" t="n">
+      <c r="N53" s="4" t="n">
         <v>192080</v>
       </c>
-      <c r="O53" s="7" t="inlineStr">
+      <c r="O53" s="5" t="inlineStr">
         <is>
           <t>Supplier assembly at 10-hour days, US$280/day (US$28/hr). 1-bed 42 hrs / 4.2 days (US$1,176). 2-bed and 3-bed 80 hrs / 8 days (US$2,240 each). Crew mix still 80% Belizean / 20% China tech — Belizeans are the standing workforce. Not in 03.03 plant hire.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+      <c r="A54" s="11" t="inlineStr">
         <is>
           <t>11.02</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B54" s="11" t="inlineStr">
         <is>
           <t>Labour &amp; duration</t>
         </is>
       </c>
-      <c r="C54" s="14" t="inlineStr">
+      <c r="C54" s="12" t="inlineStr">
         <is>
           <t>Solar PV + inverter install — local crew (man-hours / home)</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D54" s="11" t="inlineStr">
         <is>
           <t>hr</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
+      <c r="E54" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F54" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="G54" s="15" t="n">
+      <c r="G54" s="13" t="n">
         <v>19.4</v>
       </c>
-      <c r="H54" s="15" t="n">
+      <c r="H54" s="13" t="n">
         <v>19.4</v>
       </c>
-      <c r="I54" s="15" t="n">
+      <c r="I54" s="13" t="n">
         <v>19.4</v>
       </c>
-      <c r="J54" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K54" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M54" s="2" t="inlineStr">
+      <c r="J54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="N54" s="2" t="inlineStr">
+      <c r="N54" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="O54" s="14" t="inlineStr">
+      <c r="O54" s="12" t="inlineStr">
         <is>
           <t>Hours TBD. Rate EST. $19.40/hr mixed: 70% Belizean electrician @ $14 + 30% China PV tech on-site @ $32. Belizean electricians run the roofs for the 12-month campaign. One Chinese tech commissions the first kits and trains. Not in 04.02–04.04 equipment.</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" s="11" t="inlineStr">
         <is>
           <t>11.03</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B55" s="11" t="inlineStr">
         <is>
           <t>Labour &amp; duration</t>
         </is>
       </c>
-      <c r="C55" s="14" t="inlineStr">
+      <c r="C55" s="12" t="inlineStr">
         <is>
           <t>China technician attendance (trainer)</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" s="11" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E55" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F55" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="G55" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" s="2" t="n"/>
-      <c r="K55" s="2" t="n"/>
-      <c r="L55" s="2" t="n"/>
-      <c r="M55" s="2" t="inlineStr">
+      <c r="G55" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" s="11" t="n"/>
+      <c r="K55" s="11" t="n"/>
+      <c r="L55" s="11" t="n"/>
+      <c r="M55" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="N55" s="2" t="inlineStr">
+      <c r="N55" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="O55" s="14" t="inlineStr">
+      <c r="O55" s="12" t="inlineStr">
         <is>
           <t>China technician as trainer/commissioner — not the standing workforce. Belizean foremen run the site after handover. Duration TBD.</t>
         </is>
@@ -3958,7 +3758,7 @@
           <t>Labour &amp; duration</t>
         </is>
       </c>
-      <c r="C56" s="7" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>Duration — module assembly on pad</t>
         </is>
@@ -3978,190 +3778,190 @@
           <t>YES</t>
         </is>
       </c>
-      <c r="G56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K56" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L56" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M56" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N56" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O56" s="7" t="inlineStr">
+      <c r="G56" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O56" s="5" t="inlineStr">
         <is>
           <t>Calendar crew-days at 10 hours/day from the supplier assembly sheet. 1-bed 4.2 days; 2-bed and 3-bed 8 days. No dollar on this line — dollars sit on 11.01.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" s="11" t="inlineStr">
         <is>
           <t>11.05</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B57" s="11" t="inlineStr">
         <is>
           <t>Labour &amp; duration</t>
         </is>
       </c>
-      <c r="C57" s="14" t="inlineStr">
+      <c r="C57" s="12" t="inlineStr">
         <is>
           <t>Duration — solar install</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D57" s="11" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E57" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F57" s="11" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="G57" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H57" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I57" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K57" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L57" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="M57" s="2" t="inlineStr">
+      <c r="G57" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M57" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="N57" s="2" t="inlineStr">
+      <c r="N57" s="11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="O57" s="14" t="inlineStr">
+      <c r="O57" s="12" t="inlineStr">
         <is>
           <t>Calendar days for PV + inverter on the roof. Fill with 11.02 labour next week.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="21" t="inlineStr">
+      <c r="A58" s="19" t="inlineStr">
         <is>
           <t>11.06</t>
         </is>
       </c>
-      <c r="B58" s="21" t="inlineStr">
+      <c r="B58" s="19" t="inlineStr">
         <is>
           <t>Labour &amp; duration</t>
         </is>
       </c>
-      <c r="C58" s="22" t="inlineStr">
+      <c r="C58" s="20" t="inlineStr">
         <is>
           <t>FF&amp;E installation labour</t>
         </is>
       </c>
-      <c r="D58" s="21" t="inlineStr">
+      <c r="D58" s="19" t="inlineStr">
         <is>
           <t>home</t>
         </is>
       </c>
-      <c r="E58" s="21" t="inlineStr">
+      <c r="E58" s="19" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F58" s="21" t="inlineStr">
+      <c r="F58" s="19" t="inlineStr">
         <is>
           <t>NO — optional</t>
         </is>
       </c>
-      <c r="G58" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H58" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I58" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K58" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L58" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M58" s="21" t="inlineStr">
+      <c r="G58" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M58" s="19" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="N58" s="21" t="inlineStr">
+      <c r="N58" s="19" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="O58" s="22" t="inlineStr">
+      <c r="O58" s="20" t="inlineStr">
         <is>
           <t>Only if the furnished upgrade is taken.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="25" t="inlineStr">
+      <c r="A60" s="23" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B60" s="25" t="inlineStr">
+      <c r="B60" s="23" t="inlineStr">
         <is>
           <t>On-costs</t>
         </is>
       </c>
-      <c r="C60" s="25" t="n"/>
-      <c r="D60" s="25" t="n"/>
-      <c r="E60" s="25" t="n"/>
-      <c r="F60" s="25" t="n"/>
-      <c r="G60" s="25" t="n"/>
-      <c r="H60" s="25" t="n"/>
-      <c r="I60" s="25" t="n"/>
-      <c r="J60" s="25" t="n"/>
-      <c r="K60" s="25" t="n"/>
-      <c r="L60" s="25" t="n"/>
-      <c r="M60" s="25" t="n"/>
-      <c r="N60" s="25" t="n"/>
-      <c r="O60" s="25" t="n"/>
+      <c r="C60" s="23" t="n"/>
+      <c r="D60" s="23" t="n"/>
+      <c r="E60" s="23" t="n"/>
+      <c r="F60" s="23" t="n"/>
+      <c r="G60" s="23" t="n"/>
+      <c r="H60" s="23" t="n"/>
+      <c r="I60" s="23" t="n"/>
+      <c r="J60" s="23" t="n"/>
+      <c r="K60" s="23" t="n"/>
+      <c r="L60" s="23" t="n"/>
+      <c r="M60" s="23" t="n"/>
+      <c r="N60" s="23" t="n"/>
+      <c r="O60" s="23" t="n"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4174,8 +3974,8 @@
           <t>Contingency 8% on works in price</t>
         </is>
       </c>
-      <c r="M61" s="5" t="n">
-        <v>534793.5208791209</v>
+      <c r="M61" s="4" t="n">
+        <v>549931.5208791209</v>
       </c>
     </row>
     <row r="62">
@@ -4189,33 +3989,23 @@
           <t>Project management 5.5%</t>
         </is>
       </c>
-      <c r="M62" s="5" t="n">
-        <v>397084.1892527473</v>
+      <c r="M62" s="4" t="n">
+        <v>408324.1542527472</v>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
-      <c r="C63" s="9" t="inlineStr">
+      <c r="C63" s="7" t="inlineStr">
         <is>
           <t>ALL-IN UNFURNISHED — Full village, no extra civil</t>
         </is>
       </c>
-      <c r="M63" s="26" t="n">
-        <v>7616796.721120879</v>
+      <c r="M63" s="24" t="n">
+        <v>7832399.686120879</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:O47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LCASA 100 BOQ worksheet · internal</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
 
@@ -4225,13 +4015,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="70" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4242,9 +4032,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>IN the shell</t>
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>IN the KDK shell list</t>
         </is>
       </c>
     </row>
@@ -4277,7 +4067,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>NOT in the shell</t>
         </is>
@@ -4300,7 +4090,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Range / fridge (08.01). Gas stove not included.</t>
+          <t>Range / fridge (08.01).</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4104,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Slab, set, assembly labour (Div 03 + 11.01)</t>
+          <t>Slab, set, Div 11.01 assembly labour</t>
         </is>
       </c>
     </row>
@@ -4333,24 +4123,24 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>Style</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>List / home</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Net −10% / home</t>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>KDK list / home</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>After 10% campaign net</t>
         </is>
       </c>
     </row>
@@ -4363,11 +4153,11 @@
       <c r="B20" t="n">
         <v>30</v>
       </c>
-      <c r="C20" s="5" t="n">
-        <v>15850</v>
-      </c>
-      <c r="D20" s="5" t="n">
-        <v>14265</v>
+      <c r="C20" s="4" t="n">
+        <v>17435</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>15691.5</v>
       </c>
     </row>
     <row r="21">
@@ -4379,11 +4169,11 @@
       <c r="B21" t="n">
         <v>45</v>
       </c>
-      <c r="C21" s="5" t="n">
-        <v>23100</v>
-      </c>
-      <c r="D21" s="5" t="n">
-        <v>20790</v>
+      <c r="C21" s="4" t="n">
+        <v>25410</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>22869</v>
       </c>
     </row>
     <row r="22">
@@ -4395,23 +4185,28 @@
       <c r="B22" t="n">
         <v>25</v>
       </c>
-      <c r="C22" s="5" t="n">
-        <v>23500</v>
-      </c>
-      <c r="D22" s="5" t="n">
-        <v>21150</v>
+      <c r="C22" s="4" t="n">
+        <v>25850</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>23265</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>100 homes</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="n">
+        <v>2312750</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>2081475</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;LCASA 100 BOQ worksheet · internal</oddHeader>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>